<commit_message>
Tighten finance audit to four source defects
</commit_message>
<xml_diff>
--- a/finance-class/Northstar_Life_Finance_Starter.xlsx
+++ b/finance-class/Northstar_Life_Finance_Starter.xlsx
@@ -386,8 +386,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="IssueLogTable" displayName="IssueLogTable" ref="A1:H13" headerRowCount="1">
-  <autoFilter ref="A1:H13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="IssueLogTable" displayName="IssueLogTable" ref="A1:H5" headerRowCount="1">
+  <autoFilter ref="A1:H5"/>
   <tableColumns count="8">
     <tableColumn id="1" name="Issue ID"/>
     <tableColumn id="2" name="Sheet / table"/>
@@ -875,54 +875,62 @@
     <row r="7" ht="42" customHeight="1" s="17">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Favorability</t>
+          <t>Audit boundary</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Premium Revenue below plan is unfavorable. Paid Claims or Operating Expense above plan is unfavorable.</t>
+          <t>Log only true source-data defects. Green learner-output cells, blank templates or canvases, and existing DataQualityFlag warnings are expected design or evidence limitations, not source defects.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" s="17">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Cause discipline</t>
+          <t>Favorability</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>Do not infer causes from variance or detail data. Open the review notes only when instructed.</t>
+          <t>Premium Revenue below plan is unfavorable. Paid Claims or Operating Expense above plan is unfavorable.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" s="17">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Completed reference</t>
+          <t>Cause discipline</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>The instructor has a separate completed workbook for demonstration and recovery. It is not a learner input.</t>
+          <t>Do not infer causes from variance or detail data. Open the review notes only when instructed.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" s="17">
       <c r="A10" s="9" t="inlineStr">
         <is>
+          <t>Completed reference</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>The instructor has a separate completed workbook for demonstration and recovery. It is not a learner input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1" s="17">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
           <t>Change review</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>At the end, ask Copilot to summarize available change history, then inspect Review &gt; Show Changes and use Version History for recovery when available. Unsupported versions and untracked features can leave gaps.</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="42" customHeight="1" s="17">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="9" t="n"/>
     </row>
     <row r="12" ht="42" customHeight="1" s="17">
       <c r="A12" s="9" t="n"/>
@@ -1088,7 +1096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="17" min="1" max="1"/>
@@ -1147,14 +1155,6 @@
     <row r="3"/>
     <row r="4"/>
     <row r="5"/>
-    <row r="6"/>
-    <row r="7"/>
-    <row r="8"/>
-    <row r="9"/>
-    <row r="10"/>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
@@ -5359,7 +5359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="20" customWidth="1" style="17" min="1" max="1"/>
@@ -5760,7 +5760,7 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Do not compare directly with Paid Claims without naming the basis</t>
+          <t>Learner-created during class; an intentional blank is not a source-data defect</t>
         </is>
       </c>
     </row>
@@ -5826,7 +5826,7 @@
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Must equal zero before analysis</t>
+          <t>Learner-created during class; an intentional blank is not a source-data defect</t>
         </is>
       </c>
     </row>
@@ -5848,98 +5848,14 @@
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>A PASS proves arithmetic consistency, not business truth</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="40.05" customHeight="1" s="17">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>ScenarioModel</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Assumption cells</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Editable percentage changes</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>State assumptions explicitly</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="40.05" customHeight="1" s="17">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>ScenarioModel</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Loss ratio</t>
-        </is>
-      </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Projected paid claims divided by projected premium</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Scenario output, not forecast</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="40.05" customHeight="1" s="17">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t>ScenarioModel</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>Operating margin proxy</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
-        <is>
-          <t>Projected premium minus projected claims and expense</t>
-        </is>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>Simplified teaching metric, not GAAP net income</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="40.05" customHeight="1" s="17">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>MonthlyContext</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="inlineStr">
-        <is>
-          <t>LossRatio</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
-        <is>
-          <t>Actual Paid Claims divided by Actual Premium Revenue</t>
-        </is>
-      </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Context only; no causal inference</t>
-        </is>
-      </c>
-    </row>
+          <t>Learner-created during class; an intentional blank is not a source-data defect</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="40.05" customHeight="1" s="17"/>
+    <row r="24" ht="40.05" customHeight="1" s="17"/>
+    <row r="25" ht="40.05" customHeight="1" s="17"/>
+    <row r="26" ht="40.05" customHeight="1" s="17"/>
   </sheetData>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.4" bottom="0.4" header="0.5" footer="0.5"/>

</xml_diff>